<commit_message>
Add Октобър Сбор special-offers menu section (test only)
New top-level menu category with 6 event items (beers + grill) from
the POS, priced in euro. Appears first in the menu for the event.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S186"/>
+  <dimension ref="A1:S192"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="23.77734375" customWidth="1" min="1" max="1"/>
@@ -13101,6 +13101,342 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>shoferhofer_500</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>october_sbor</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>special_offers</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>schofferhofer</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>wheat_beer</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Шьоферхофер 0,5 л</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Schöfferhofer 0,5 l</t>
+        </is>
+      </c>
+      <c r="J187" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="K187" t="n">
+        <v>500</v>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="N187" t="b">
+        <v>0</v>
+      </c>
+      <c r="O187" t="b">
+        <v>0</v>
+      </c>
+      <c r="P187" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q187" t="b">
+        <v>1</v>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>alcohol</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>san_migel_1000</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>october_sbor</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>special_offers</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>san_miguel</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>lager</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Сан Мигел 1 л</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>San Miguel 1 l</t>
+        </is>
+      </c>
+      <c r="J188" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="K188" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="N188" t="b">
+        <v>0</v>
+      </c>
+      <c r="O188" t="b">
+        <v>0</v>
+      </c>
+      <c r="P188" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q188" t="b">
+        <v>1</v>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>alcohol</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>benediktiner_bure_5l</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>october_sbor</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>special_offers</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>benediktiner</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>wheat_beer</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Бенедиктер буре 5 л</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Benediktiner keg 5 l</t>
+        </is>
+      </c>
+      <c r="J189" t="n">
+        <v>39</v>
+      </c>
+      <c r="K189" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="N189" t="b">
+        <v>0</v>
+      </c>
+      <c r="O189" t="b">
+        <v>0</v>
+      </c>
+      <c r="P189" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q189" t="b">
+        <v>1</v>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>alcohol</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>meshana_skara_sbor</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>october_sbor</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>special_offers</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Мешана скара</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Mixed grill</t>
+        </is>
+      </c>
+      <c r="J190" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="N190" t="b">
+        <v>0</v>
+      </c>
+      <c r="O190" t="b">
+        <v>0</v>
+      </c>
+      <c r="P190" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q190" t="b">
+        <v>1</v>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>kebapche_sbor</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>october_sbor</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>special_offers</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Кебапче</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Kebapche</t>
+        </is>
+      </c>
+      <c r="J191" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N191" t="b">
+        <v>0</v>
+      </c>
+      <c r="O191" t="b">
+        <v>0</v>
+      </c>
+      <c r="P191" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q191" t="b">
+        <v>1</v>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>kyufte_sbor</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>october_sbor</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>special_offers</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Кюфте</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Kyufte</t>
+        </is>
+      </c>
+      <c r="J192" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N192" t="b">
+        <v>0</v>
+      </c>
+      <c r="O192" t="b">
+        <v>0</v>
+      </c>
+      <c r="P192" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q192" t="b">
+        <v>1</v>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Reorder the Октобър Сбор items: beers first, kitchen last
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -13169,7 +13169,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>san_migel_1000</t>
+          <t>benediktiner_500</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -13184,29 +13184,29 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>san_miguel</t>
+          <t>benediktiner</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>lager</t>
+          <t>wheat_beer</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Сан Мигел 1 л</t>
+          <t>Бенедиктер 0,5 л</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>San Miguel 1 l</t>
+          <t>Benediktiner 0,5 l</t>
         </is>
       </c>
       <c r="J188" t="n">
-        <v>7.4</v>
+        <v>4.2</v>
       </c>
       <c r="K188" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -13234,7 +13234,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>benediktiner_bure_5l</t>
+          <t>san_migel_1000</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -13249,29 +13249,29 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>benediktiner</t>
+          <t>san_miguel</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>wheat_beer</t>
+          <t>lager</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Бенедиктер буре 5 л</t>
+          <t>Сан Мигел 1 л</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Benediktiner keg 5 l</t>
+          <t>San Miguel 1 l</t>
         </is>
       </c>
       <c r="J189" t="n">
-        <v>39</v>
+        <v>7.4</v>
       </c>
       <c r="K189" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
       <c r="L189" t="inlineStr">
         <is>
@@ -13299,7 +13299,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>meshana_skara_sbor</t>
+          <t>benediktiner_bure_5l</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -13312,18 +13312,36 @@
           <t>special_offers</t>
         </is>
       </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>benediktiner</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>wheat_beer</t>
+        </is>
+      </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Мешана скара</t>
+          <t>Бенедиктер буре 5 л</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Mixed grill</t>
+          <t>Benediktiner keg 5 l</t>
         </is>
       </c>
       <c r="J190" t="n">
-        <v>9.5</v>
+        <v>39</v>
+      </c>
+      <c r="K190" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
       </c>
       <c r="N190" t="b">
         <v>0</v>
@@ -13339,14 +13357,14 @@
       </c>
       <c r="R190" t="inlineStr">
         <is>
-          <t>food</t>
+          <t>alcohol</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>kebapche_sbor</t>
+          <t>meshana_skara_sbor</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -13361,16 +13379,16 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Кебапче</t>
+          <t>Мешана скара</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Kebapche</t>
+          <t>Mixed grill</t>
         </is>
       </c>
       <c r="J191" t="n">
-        <v>1.5</v>
+        <v>9.5</v>
       </c>
       <c r="N191" t="b">
         <v>0</v>
@@ -13393,7 +13411,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>kyufte_sbor</t>
+          <t>kebapche_sbor</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -13408,12 +13426,12 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Кюфте</t>
+          <t>Кебапче</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Kyufte</t>
+          <t>Kebapche</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -13440,7 +13458,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>benediktiner_500</t>
+          <t>kyufte_sbor</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -13453,36 +13471,18 @@
           <t>special_offers</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>benediktiner</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>wheat_beer</t>
-        </is>
-      </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Бенедиктер 0,5 л</t>
+          <t>Кюфте</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Benediktiner 0,5 l</t>
+          <t>Kyufte</t>
         </is>
       </c>
       <c r="J193" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="K193" t="n">
-        <v>500</v>
-      </c>
-      <c r="L193" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
+        <v>1.5</v>
       </c>
       <c r="N193" t="b">
         <v>0</v>
@@ -13498,7 +13498,7 @@
       </c>
       <c r="R193" t="inlineStr">
         <is>
-          <t>alcohol</t>
+          <t>food</t>
         </is>
       </c>
     </row>

</xml_diff>